<commit_message>
Harden APMM submission and add end-to-end tests
</commit_message>
<xml_diff>
--- a/outputs/fRL_winners.xlsx
+++ b/outputs/fRL_winners.xlsx
@@ -69,7 +69,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
@@ -83,6 +83,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -460,7 +463,7 @@
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="42" customWidth="1" min="6" max="6"/>
+    <col width="48" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="17" customWidth="1" min="8" max="8"/>
     <col width="21" customWidth="1" min="9" max="9"/>
@@ -472,7 +475,7 @@
     <col width="16" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="24" customHeight="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
           <t>Source</t>
@@ -575,7 +578,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F2" s="4" t="inlineStr">
+      <c r="F2" s="6" t="inlineStr">
         <is>
           <t>Infosquare global Solutions</t>
         </is>
@@ -609,10 +612,10 @@
       <c r="M2" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="N2" s="6" t="n">
+      <c r="N2" s="7" t="n">
         <v>46044</v>
       </c>
-      <c r="O2" s="6" t="n">
+      <c r="O2" s="7" t="n">
         <v>47119</v>
       </c>
     </row>
@@ -642,7 +645,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F3" s="4" t="inlineStr">
+      <c r="F3" s="6" t="inlineStr">
         <is>
           <t>Best infosystems Ltd.</t>
         </is>
@@ -676,14 +679,14 @@
       <c r="M3" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="N3" s="6" t="n">
+      <c r="N3" s="7" t="n">
         <v>45813</v>
       </c>
-      <c r="O3" s="6" t="n">
+      <c r="O3" s="7" t="n">
         <v>46177</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" ht="32" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
           <t>Purchase</t>
@@ -709,7 +712,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F4" s="4" t="inlineStr">
+      <c r="F4" s="6" t="inlineStr">
         <is>
           <t>Vinay Kumar Gedhela (Proprietor of Trillinium Organisation)</t>
         </is>
@@ -743,10 +746,10 @@
       <c r="M4" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="N4" s="6" t="n">
+      <c r="N4" s="7" t="n">
         <v>46052</v>
       </c>
-      <c r="O4" s="6" t="n">
+      <c r="O4" s="7" t="n">
         <v>46417</v>
       </c>
     </row>
@@ -776,7 +779,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr">
+      <c r="F5" s="6" t="inlineStr">
         <is>
           <t>Direction</t>
         </is>
@@ -810,10 +813,10 @@
       <c r="M5" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="N5" s="6" t="n">
+      <c r="N5" s="7" t="n">
         <v>45839</v>
       </c>
-      <c r="O5" s="6" t="n">
+      <c r="O5" s="7" t="n">
         <v>46568</v>
       </c>
     </row>
@@ -843,7 +846,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F6" s="4" t="inlineStr">
+      <c r="F6" s="6" t="inlineStr">
         <is>
           <t>Spectral Consultants</t>
         </is>
@@ -877,10 +880,10 @@
       <c r="M6" s="5" t="n">
         <v>29</v>
       </c>
-      <c r="N6" s="6" t="n">
+      <c r="N6" s="7" t="n">
         <v>45987</v>
       </c>
-      <c r="O6" s="6" t="n">
+      <c r="O6" s="7" t="n">
         <v>46352</v>
       </c>
     </row>
@@ -910,7 +913,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F7" s="4" t="inlineStr">
+      <c r="F7" s="6" t="inlineStr">
         <is>
           <t>Infosys Limited</t>
         </is>
@@ -940,14 +943,14 @@
       <c r="M7" s="5" t="n">
         <v>1133</v>
       </c>
-      <c r="N7" s="6" t="n">
+      <c r="N7" s="7" t="n">
         <v>45464</v>
       </c>
-      <c r="O7" s="6" t="n">
+      <c r="O7" s="7" t="n">
         <v>46552</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" ht="32" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
           <t>Purchase</t>
@@ -969,7 +972,7 @@
       <c r="E8" s="5" t="n">
         <v>30798</v>
       </c>
-      <c r="F8" s="4" t="inlineStr">
+      <c r="F8" s="6" t="inlineStr">
         <is>
           <t>Parikshit Naramdeo (Proprietor of Orange Wings Recruitment Services)</t>
         </is>
@@ -1003,14 +1006,14 @@
       <c r="M8" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="N8" s="6" t="n">
+      <c r="N8" s="7" t="n">
         <v>45972</v>
       </c>
-      <c r="O8" s="6" t="n">
+      <c r="O8" s="7" t="n">
         <v>47067</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" ht="32" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
           <t>Purchase</t>
@@ -1032,7 +1035,7 @@
       <c r="E9" s="5" t="n">
         <v>24219</v>
       </c>
-      <c r="F9" s="4" t="inlineStr">
+      <c r="F9" s="6" t="inlineStr">
         <is>
           <t>Seharish Khulud (Proprietor of Digital Concept Solutions)</t>
         </is>
@@ -1066,10 +1069,10 @@
       <c r="M9" s="5" t="n">
         <v>15</v>
       </c>
-      <c r="N9" s="6" t="n">
+      <c r="N9" s="7" t="n">
         <v>45958</v>
       </c>
-      <c r="O9" s="6" t="n">
+      <c r="O9" s="7" t="n">
         <v>46323</v>
       </c>
     </row>
@@ -1095,7 +1098,7 @@
       <c r="E10" s="5" t="n">
         <v>20038</v>
       </c>
-      <c r="F10" s="4" t="inlineStr">
+      <c r="F10" s="6" t="inlineStr">
         <is>
           <t>Advantum Health Private Limited</t>
         </is>
@@ -1129,10 +1132,10 @@
       <c r="M10" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="N10" s="6" t="n">
+      <c r="N10" s="7" t="n">
         <v>45981</v>
       </c>
-      <c r="O10" s="6" t="n">
+      <c r="O10" s="7" t="n">
         <v>46073</v>
       </c>
     </row>
@@ -1158,7 +1161,7 @@
       <c r="E11" s="5" t="n">
         <v>19829</v>
       </c>
-      <c r="F11" s="4" t="inlineStr">
+      <c r="F11" s="6" t="inlineStr">
         <is>
           <t>Reba Financial Services</t>
         </is>
@@ -1192,10 +1195,10 @@
       <c r="M11" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="N11" s="6" t="n">
+      <c r="N11" s="7" t="n">
         <v>45996</v>
       </c>
-      <c r="O11" s="6" t="n">
+      <c r="O11" s="7" t="n">
         <v>46085</v>
       </c>
     </row>
@@ -1221,7 +1224,7 @@
       <c r="E12" s="5" t="n">
         <v>12635</v>
       </c>
-      <c r="F12" s="4" t="inlineStr">
+      <c r="F12" s="6" t="inlineStr">
         <is>
           <t>Izee Manpower Consultancy Private Limited</t>
         </is>
@@ -1255,10 +1258,10 @@
       <c r="M12" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="N12" s="6" t="n">
+      <c r="N12" s="7" t="n">
         <v>45987</v>
       </c>
-      <c r="O12" s="6" t="n">
+      <c r="O12" s="7" t="n">
         <v>46352</v>
       </c>
     </row>
@@ -1284,7 +1287,7 @@
       <c r="E13" s="5" t="n">
         <v>57519</v>
       </c>
-      <c r="F13" s="4" t="inlineStr">
+      <c r="F13" s="6" t="inlineStr">
         <is>
           <t>Icici Bank Limited</t>
         </is>
@@ -1318,10 +1321,10 @@
       <c r="M13" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="N13" s="6" t="n">
+      <c r="N13" s="7" t="n">
         <v>45749</v>
       </c>
-      <c r="O13" s="6" t="n">
+      <c r="O13" s="7" t="n">
         <v>46113</v>
       </c>
     </row>
@@ -1347,7 +1350,7 @@
       <c r="E14" s="5" t="n">
         <v>53756</v>
       </c>
-      <c r="F14" s="4" t="inlineStr">
+      <c r="F14" s="6" t="inlineStr">
         <is>
           <t>LTIMindtree Limited</t>
         </is>
@@ -1381,10 +1384,10 @@
       <c r="M14" s="5" t="n">
         <v>86</v>
       </c>
-      <c r="N14" s="6" t="n">
+      <c r="N14" s="7" t="n">
         <v>45490</v>
       </c>
-      <c r="O14" s="6" t="n">
+      <c r="O14" s="7" t="n">
         <v>46585</v>
       </c>
     </row>
@@ -1410,7 +1413,7 @@
       <c r="E15" s="5" t="n">
         <v>47160</v>
       </c>
-      <c r="F15" s="4" t="inlineStr">
+      <c r="F15" s="6" t="inlineStr">
         <is>
           <t>Certzine Recruitment Solutions</t>
         </is>
@@ -1444,14 +1447,14 @@
       <c r="M15" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="N15" s="6" t="n">
+      <c r="N15" s="7" t="n">
         <v>45594</v>
       </c>
-      <c r="O15" s="6" t="n">
+      <c r="O15" s="7" t="n">
         <v>46684</v>
       </c>
     </row>
-    <row r="16">
+    <row r="16" ht="32" customHeight="1">
       <c r="A16" s="4" t="inlineStr">
         <is>
           <t>Purchase</t>
@@ -1473,7 +1476,7 @@
       <c r="E16" s="5" t="n">
         <v>45146</v>
       </c>
-      <c r="F16" s="4" t="inlineStr">
+      <c r="F16" s="6" t="inlineStr">
         <is>
           <t>Rahul Kishorechandra Ganatra (Proprietor of R K Placements)</t>
         </is>
@@ -1507,10 +1510,10 @@
       <c r="M16" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="N16" s="6" t="n">
+      <c r="N16" s="7" t="n">
         <v>45749</v>
       </c>
-      <c r="O16" s="6" t="n">
+      <c r="O16" s="7" t="n">
         <v>46112</v>
       </c>
     </row>
@@ -1536,7 +1539,7 @@
       <c r="E17" s="5" t="n">
         <v>45145</v>
       </c>
-      <c r="F17" s="4" t="inlineStr">
+      <c r="F17" s="6" t="inlineStr">
         <is>
           <t>BR Raysoft Global Private Limited</t>
         </is>
@@ -1570,10 +1573,10 @@
       <c r="M17" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="N17" s="6" t="n">
+      <c r="N17" s="7" t="n">
         <v>45855</v>
       </c>
-      <c r="O17" s="6" t="n">
+      <c r="O17" s="7" t="n">
         <v>46219</v>
       </c>
     </row>

</xml_diff>